<commit_message>
Move MOD1 and MOD2 training steps to LMOC.
</commit_message>
<xml_diff>
--- a/HX/Authorization Process Flow.xlsx
+++ b/HX/Authorization Process Flow.xlsx
@@ -900,7 +900,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N52"/>
+  <dimension ref="A1:L52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9.140625" customWidth="1" style="1" min="1" max="1"/>
@@ -1624,7 +1624,7 @@
       </c>
       <c r="F15" s="17" t="inlineStr">
         <is>
-          <t>HX Certifiers</t>
+          <t>HX LMOC</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1672,7 +1672,7 @@
       </c>
       <c r="F16" s="17" t="inlineStr">
         <is>
-          <t>HX Certifiers</t>
+          <t>HX LMOC</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -3138,7 +3138,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>HX Certifiers</t>
+          <t>HX LMOC</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -3186,7 +3186,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>HX Certifiers</t>
+          <t>HX LMOC</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">

</xml_diff>